<commit_message>
Severity policy: every confusing error is Cao; only SEO length/format and SKU characters are Thap
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0149ELLgZdjaY7wRsdGLp26m
</commit_message>
<xml_diff>
--- a/listing-monitor/reports/2026-10-30/qa_2026-10-30.xlsx
+++ b/listing-monitor/reports/2026-10-30/qa_2026-10-30.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'KFK'!$A$1:$N$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RFK'!$A$1:$N$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RFK'!$A$1:$N$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CFS'!$A$1:$N$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -63,17 +63,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2E3E5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
   </fills>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -488,7 +488,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tạo lúc 2026-10-30 23:29. Mức độ: Cao = sai thông tin / gây confuse khách và Google; Trung bình = cần sửa; Thấp = nên sửa.</t>
+          <t>Tạo lúc 2026-10-31 18:34. Mức độ: Cao = phải fix (mọi lỗi gây confuse khách / AI / Google); Cần xác nhận = cần người xem; Thấp = fix sau (độ dài SEO title/meta, ký tự SKU).</t>
         </is>
       </c>
     </row>
@@ -515,17 +515,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Lỗi Cao</t>
+          <t>Lỗi Cao (phải fix)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Lỗi Trung bình</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Lỗi Thấp</t>
+          <t>Lỗi Thấp (fix sau)</t>
         </is>
       </c>
     </row>
@@ -542,16 +542,16 @@
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -567,16 +567,16 @@
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="F6" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -592,16 +592,16 @@
         <v>11</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="G7" t="n">
-        <v>34</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -643,20 +643,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sai cầu thủ</t>
+          <t>Category / Tag</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>0</v>
       </c>
       <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="D11" t="n">
-        <v>1</v>
-      </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -700,7 +700,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sai season</t>
+          <t>Sai cầu thủ</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -719,17 +719,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sai đối tượng</t>
+          <t>Sai season</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>0</v>
       </c>
       <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
         <v>1</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
       </c>
       <c r="E15" t="n">
         <v>1</v>
@@ -738,83 +738,83 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>Sai đối tượng</t>
         </is>
       </c>
       <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
         <v>1</v>
       </c>
-      <c r="C16" t="n">
-        <v>2</v>
-      </c>
       <c r="D16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C17" t="n">
         <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Words to Avoid</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Club bị report</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C19" t="n">
         <v>2</v>
       </c>
       <c r="D19" t="n">
+        <v>5</v>
+      </c>
+      <c r="E19" t="n">
         <v>7</v>
-      </c>
-      <c r="E19" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Club bị report</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -824,70 +824,89 @@
         <v>2</v>
       </c>
       <c r="D20" t="n">
+        <v>7</v>
+      </c>
+      <c r="E20" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
         <v>5</v>
       </c>
-      <c r="E20" t="n">
+      <c r="E21" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Lỗi lặp lại trên phần lớn listing của 1 site (nhiều khả năng do TEMPLATE, sửa template 1 lần)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Site</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Nhóm</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Vị trí</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Lỗi</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Số listing</t>
         </is>
       </c>
-      <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>CFS</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Club bị report</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Ảnh</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Barcelona</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>7/13</t>
         </is>
@@ -998,7 +1017,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1056,7 +1075,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1079,22 +1098,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Club bị report</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 67 ký tự (nên &lt;= 60)</t>
+          <t>Barcelona (Nike): sheet ghi KFK 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -1114,7 +1133,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1137,22 +1156,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Club bị report</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Barcelona (Nike): sheet ghi KFK 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
+          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Check blur logo</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -1170,7 +1189,7 @@
       <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -1195,22 +1214,22 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>SKU (Google)</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>SKU 'KFK_BA_TH_KD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>SEO title dài 67 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -1228,7 +1247,7 @@
       <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -1253,22 +1272,22 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>SKU (Google)</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
+          <t>SKU 'KFK_BA_TH_KD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Cần người check</t>
+          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -1309,7 +1328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1403,7 +1422,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1461,7 +1480,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1519,7 +1538,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1577,7 +1596,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1600,22 +1619,22 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Category / Tag</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>SKU variation</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>SKU cha RFK_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27 nhưng variation mang SKU khác đầu: RFK_BARRM_HOGP1_KD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27_28 (12-13 yrs) (+13)</t>
+          <t>Category đội tuyển 'Spain' nhưng tên sản phẩm không có Spain</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Sửa SKU variation theo SKU cha (clone quên đổi)</t>
+          <t>Bỏ category 'Spain' (chỉ dùng cho sản phẩm của đội tuyển Spain)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -1635,7 +1654,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1658,22 +1677,22 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>SKU variation</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Option "Add combo badges for 2 items only:" không ghi tên giải (ảnh/gợi ý: La Liga (champion), La Liga).</t>
+          <t>SKU cha RFK_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27 nhưng variation mang SKU khác đầu: RFK_BARRM_HOGP1_KD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27_28 (12-13 yrs) (+13)</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Ghi tên giải vào tên option (vd 'Add Premier League Badge')</t>
+          <t>Sửa SKU variation theo SKU cha (clone quên đổi)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -1693,51 +1712,51 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-30 10:04</t>
+          <t>2026-10-30 09:01</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>132430</v>
+        <v>132408</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>RFK_BARRM_HOGP_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
+          <t>RFK_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Shirt Gift Set – Home Kids Football Shirts</t>
+          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Kit Gift Set – Home Kids Football Kits (With Socks)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>'Features the' (...0 Barcelona Home Men’s Shirt: Features the iconic blue and red vertical ...); 'worldwide' (...tity that resonates with fans worldwide. Its commitment to exciting f...)</t>
+          <t>Option "Add combo badges for 2 items only:" không ghi tên giải (ảnh/gợi ý: La Liga (champion), La Liga).</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Features the -&gt; includes the / highlights the; worldwide -&gt; (bỏ)</t>
+          <t>Ghi tên giải vào tên option (vd 'Add Premier League Badge')</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-shirt-gift-set-home-kids-football-shirts/</t>
+          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-kit-gift-set-home-kids-football-kits-with-socks/</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
@@ -1751,7 +1770,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1774,22 +1793,22 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>Sai đối tượng</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Short description</t>
+          <t>Tên sản phẩm</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
+          <t>SKU 'AD' (Men/Adult) nhưng tên ghi Kids</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
+          <t>Sửa tên hoặc SKU cho khớp</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
@@ -1809,7 +1828,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1832,22 +1851,22 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Words to Avoid</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>SKU variation</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>SKU cha RFK_BARRM_HOGP_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27 nhưng variation mang SKU khác đầu: RFK_BARRM_HOGP2_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27_XL (+9)</t>
+          <t>'Features the' (...0 Barcelona Home Men’s Shirt: Features the iconic blue and red vertical ...); 'worldwide' (...tity that resonates with fans worldwide. Its commitment to exciting f...)</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Sửa SKU variation theo SKU cha (clone quên đổi)</t>
+          <t>Features the -&gt; includes the / highlights the; worldwide -&gt; (bỏ)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -1867,7 +1886,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1890,22 +1909,22 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Sai đối tượng</t>
+          <t>Words to Avoid</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Attribute Gender Age</t>
+          <t>Short description</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Tên có Kids nhưng Gender Age = "Men"</t>
+          <t>'Trustpilot' (★ Rated 4.8/5 on Trustpilot ★★★★★ £ Best-Value Prices Pre...)</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Sửa Gender Age</t>
+          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -1925,7 +1944,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1948,22 +1967,22 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>Size chart</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Option "Add combo badges for 2 items only:" không ghi tên giải (ảnh/gợi ý: La Liga (champion), La Liga).</t>
+          <t>Listing Men/Adult nhưng dùng size chart Kids (Replica-Football-Kits-Kid_s-Kit-Size-Chart.png)</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Ghi tên giải vào tên option (vd 'Add Premier League Badge')</t>
+          <t>Đổi size chart đúng đối tượng</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -1981,53 +2000,53 @@
       <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-30 09:01</t>
+          <t>2026-10-30 10:04</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>132408</v>
+        <v>132430</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>RFK_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
+          <t>RFK_BARRM_HOGP_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Kit Gift Set – Home Kids Football Kits (With Socks)</t>
+          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Shirt Gift Set – Home Kids Football Shirts</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Category / Tag</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Season trong SKU ghi '2026/27', các SKU khác ghi '26/27'</t>
+          <t>Category đội tuyển 'Spain' nhưng tên sản phẩm không có Spain</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Đổi thành 26/27</t>
+          <t>Bỏ category 'Spain' (chỉ dùng cho sản phẩm của đội tuyển Spain)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-kit-gift-set-home-kids-football-kits-with-socks/</t>
+          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-shirt-gift-set-home-kids-football-shirts/</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -2039,53 +2058,53 @@
       <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-10-30 09:01</t>
+          <t>2026-10-30 10:04</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>132408</v>
+        <v>132430</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>RFK_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
+          <t>RFK_BARRM_HOGP_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Kit Gift Set – Home Kids Football Kits (With Socks)</t>
+          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Shirt Gift Set – Home Kids Football Shirts</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>SKU variation</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 147 ký tự (nên &lt;= 60)</t>
+          <t>SKU cha RFK_BARRM_HOGP_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27 nhưng variation mang SKU khác đầu: RFK_BARRM_HOGP2_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27_XL (+9)</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Sửa SKU variation theo SKU cha (clone quên đổi)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-kit-gift-set-home-kids-football-kits-with-socks/</t>
+          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-shirt-gift-set-home-kids-football-shirts/</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
@@ -2097,53 +2116,53 @@
       <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-30 09:01</t>
+          <t>2026-10-30 10:04</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>132408</v>
+        <v>132430</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>RFK_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
+          <t>RFK_BARRM_HOGP_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Kit Gift Set – Home Kids Football Kits (With Socks)</t>
+          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Shirt Gift Set – Home Kids Football Shirts</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Club bị report</t>
+          <t>Sai đối tượng</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Attribute Gender Age</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Barcelona (Nike): sheet ghi RFK 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
+          <t>Tên có Kids nhưng Gender Age = "Men"</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Check blur logo</t>
+          <t>Sửa Gender Age</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-kit-gift-set-home-kids-football-kits-with-socks/</t>
+          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-shirt-gift-set-home-kids-football-shirts/</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -2155,53 +2174,53 @@
       <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-30 09:01</t>
+          <t>2026-10-30 10:04</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>132408</v>
+        <v>132430</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>RFK_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
+          <t>RFK_BARRM_HOGP_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Kit Gift Set – Home Kids Football Kits (With Socks)</t>
+          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Shirt Gift Set – Home Kids Football Shirts</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>SKU (Google)</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>SKU 'RFK_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>Option "Add combo badges for 2 items only:" không ghi tên giải (ảnh/gợi ý: La Liga (champion), La Liga).</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+          <t>Ghi tên giải vào tên option (vd 'Add Premier League Badge')</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-kit-gift-set-home-kids-football-kits-with-socks/</t>
+          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-shirt-gift-set-home-kids-football-shirts/</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -2215,7 +2234,7 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2238,22 +2257,22 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>Club bị report</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
+          <t>Barcelona (Nike): sheet ghi RFK 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>Cần người check</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -2273,51 +2292,51 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-10-30 10:04</t>
+          <t>2026-10-30 09:01</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>132430</v>
+        <v>132408</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>RFK_BARRM_HOGP_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
+          <t>RFK_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Shirt Gift Set – Home Kids Football Shirts</t>
+          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Kit Gift Set – Home Kids Football Kits (With Socks)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Season trong SKU ghi '2026/27', các SKU khác ghi '26/27'</t>
+          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Đổi thành 26/27</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-shirt-gift-set-home-kids-football-shirts/</t>
+          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-kit-gift-set-home-kids-football-kits-with-socks/</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
@@ -2331,7 +2350,7 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2354,22 +2373,22 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Club bị report</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 138 ký tự (nên &lt;= 60)</t>
+          <t>Barcelona (Nike): sheet ghi RFK 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -2389,7 +2408,7 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2412,22 +2431,22 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Club bị report</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Barcelona (Nike): sheet ghi RFK 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
+          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Check blur logo</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -2445,27 +2464,27 @@
       <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-30 10:04</t>
+          <t>2026-10-30 09:01</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>132430</v>
+        <v>132408</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>RFK_BARRM_HOGP_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
+          <t>RFK_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Shirt Gift Set – Home Kids Football Shirts</t>
+          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Kit Gift Set – Home Kids Football Kits (With Socks)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2475,23 +2494,23 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>SKU (Google)</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>SKU 'RFK_BARRM_HOGP_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>Season trong SKU ghi '2026/27', các SKU khác ghi '26/27'</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+          <t>Đổi thành 26/27</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-shirt-gift-set-home-kids-football-shirts/</t>
+          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-kit-gift-set-home-kids-football-kits-with-socks/</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -2503,53 +2522,53 @@
       <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-30 10:04</t>
+          <t>2026-10-30 09:01</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>132430</v>
+        <v>132408</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>RFK_BARRM_HOGP_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
+          <t>RFK_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Shirt Gift Set – Home Kids Football Shirts</t>
+          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Kit Gift Set – Home Kids Football Kits (With Socks)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
+          <t>SEO title dài 147 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Cần người check</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-shirt-gift-set-home-kids-football-shirts/</t>
+          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-kit-gift-set-home-kids-football-kits-with-socks/</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2560,8 +2579,240 @@
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
     </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-10-30 09:01</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>132408</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>RFK_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Kit Gift Set – Home Kids Football Kits (With Socks)</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>SKU (Google)</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>SKU 'RFK_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-kit-gift-set-home-kids-football-kits-with-socks/</t>
+        </is>
+      </c>
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-10-30 10:04</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>132430</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>RFK_BARRM_HOGP_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Shirt Gift Set – Home Kids Football Shirts</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Season trong SKU ghi '2026/27', các SKU khác ghi '26/27'</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>Đổi thành 26/27</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-shirt-gift-set-home-kids-football-shirts/</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-10-30 10:04</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>132430</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>RFK_BARRM_HOGP_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Shirt Gift Set – Home Kids Football Shirts</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>SEO title</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>SEO title dài 138 ký tự (nên &lt;= 60)</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-shirt-gift-set-home-kids-football-shirts/</t>
+        </is>
+      </c>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-10-30 10:04</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>132430</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>RFK_BARRM_HOGP_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Barcelona and Real Madrid LAMINE YAMAL 10 and MBAPPÉ 10 2026/27 Full Shirt Gift Set – Home Kids Football Shirts</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>SKU (Google)</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>SKU 'RFK_BARRM_HOGP_AD_LAMINE YAMAL 10 MBAPPÉ 10_2026/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>https://replicafootballkits.com/product/brclna-and-rl-md-lamine-yamal-10-and-mbappe-10-2026-27-full-shirt-gift-set-home-kids-football-shirts/</t>
+        </is>
+      </c>
+      <c r="L25" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N21"/>
+  <autoFilter ref="A1:N25"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
@@ -2603,6 +2854,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2706,53 +2965,53 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Cao</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-30 15:09</t>
+          <t>2026-10-30 03:22</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>85690</v>
+        <v>85634</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CFS_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_26/27</t>
+          <t>CFS_BAR_AW_AD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Barcelona and Real Madrid 2026/27 Gift Pack – Home Kids Cheap Football Kits – LAMINE YAMAL 10 and MBAPPÉ 10 (With socks)</t>
+          <t>Barcelona GORDON 17 Away Men Cheap Football Shirt 2026/27</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Sai cầu thủ</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Trang sản phẩm (option / tab / description)</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>Listing in sẵn LAMINE YAMAL 10 MBAPPÉ 10 nhưng trang vẫn cho/nhắc personalise: "Personalisation for 2 items only £16"</t>
+          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Bỏ option / đoạn personalisation trên listing in sẵn</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-and-real-madrid-2026-27-gift-pack-home-kids-cheap-football-kits-lamine-yamal-10-and-mbappe-10/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-away-men-cheap-football-shirt-2026-27/</t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
@@ -2766,51 +3025,51 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-30 15:09</t>
+          <t>2026-10-30 03:27</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>85690</v>
+        <v>85642</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CFS_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_26/27</t>
+          <t>CFS_BAR_AW_KD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Barcelona and Real Madrid 2026/27 Gift Pack – Home Kids Cheap Football Kits – LAMINE YAMAL 10 and MBAPPÉ 10 (With socks)</t>
+          <t>Barcelona GORDON 17 Away Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sai season</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Ảnh / alt text</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>1 ảnh có alt ghi season khác (vd: "Real Madrid and Barcelona 2025/26 Gift Pack - Home Kids Cheap Football Kits - MBAPPÉ 10 and LAMINE YAMAL 10 (With Socks)")</t>
+          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Sửa alt text / kiểm tra ảnh</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-and-real-madrid-2026-27-gift-pack-home-kids-cheap-football-kits-lamine-yamal-10-and-mbappe-10/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-away-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -2824,51 +3083,51 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-30 15:09</t>
+          <t>2026-10-30 03:31</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>85690</v>
+        <v>85652</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CFS_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_26/27</t>
+          <t>CFS_BAR_HO_AD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Barcelona and Real Madrid 2026/27 Gift Pack – Home Kids Cheap Football Kits – LAMINE YAMAL 10 and MBAPPÉ 10 (With socks)</t>
+          <t>Barcelona GORDON 17 Home Men Cheap Football Shirt 2026/27</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>SKU variation</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>SKU cha CFS_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_26/27 nhưng variation mang SKU khác đầu: CFS_BARRM1_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_26/27_16 (3-4 yrs) (+6)</t>
+          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Sửa SKU variation theo SKU cha (clone quên đổi)</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-and-real-madrid-2026-27-gift-pack-home-kids-cheap-football-kits-lamine-yamal-10-and-mbappe-10/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-home-men-cheap-football-shirt-2026-27/</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -2880,53 +3139,53 @@
       <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-30 01:52</t>
+          <t>2026-10-30 03:35</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>85593</v>
+        <v>85660</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CFS_ARG_AWLV_AD_MARADONA 10_1994</t>
+          <t>CFS_BAR_HO_KD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Retro Argentina MARADONA 10 Away Men Cheap Football Shirt 1994 Long Sleeve</t>
+          <t>Barcelona GORDON 17 Home Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 74 ký tự (nên &lt;= 60)</t>
+          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/retro-argentina-maradona-10-away-men-cheap-football-shirt-1994-long-sleeve/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-home-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
@@ -2938,53 +3197,53 @@
       <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-30 01:52</t>
+          <t>2026-10-30 03:39</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>85593</v>
+        <v>85670</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CFS_ARG_AWLV_AD_MARADONA 10_1994</t>
+          <t>CFS_BAR_TH_AD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Retro Argentina MARADONA 10 Away Men Cheap Football Shirt 1994 Long Sleeve</t>
+          <t>Barcelona GORDON 17 Third Men Cheap Football Shirt 2026/27</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>SKU (Google)</t>
+          <t>Số lượng ảnh</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>SKU 'CFS_ARG_AWLV_AD_MARADONA 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+          <t>Thêm ảnh</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/retro-argentina-maradona-10-away-men-cheap-football-shirt-1994-long-sleeve/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-third-men-cheap-football-shirt-2026-27/</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -2996,53 +3255,53 @@
       <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-30 02:02</t>
+          <t>2026-10-30 15:09</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>85602</v>
+        <v>85690</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CFS_ARG_AWLV_KD_MARADONA 10_1994</t>
+          <t>CFS_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_26/27</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Retro Argentina MARADONA 10 Away Kids Cheap Football Kit 1994 Long Sleeve</t>
+          <t>Barcelona and Real Madrid 2026/27 Gift Pack – Home Kids Cheap Football Kits – LAMINE YAMAL 10 and MBAPPÉ 10 (With socks)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Sai season</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Ảnh / alt text</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 73 ký tự (nên &lt;= 60)</t>
+          <t>1 ảnh có alt ghi season khác (vd: "Real Madrid and Barcelona 2025/26 Gift Pack - Home Kids Cheap Football Kits - MBAPPÉ 10 and LAMINE YAMAL 10 (With Socks)")</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Sửa alt text / kiểm tra ảnh</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/retro-argentina-maradona-10-away-kids-cheap-football-kit-1994-long-sleeve/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-and-real-madrid-2026-27-gift-pack-home-kids-cheap-football-kits-lamine-yamal-10-and-mbappe-10/</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
@@ -3054,27 +3313,27 @@
       <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-30 02:02</t>
+          <t>2026-10-30 15:09</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>85602</v>
+        <v>85690</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CFS_ARG_AWLV_KD_MARADONA 10_1994</t>
+          <t>CFS_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_26/27</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Retro Argentina MARADONA 10 Away Kids Cheap Football Kit 1994 Long Sleeve</t>
+          <t>Barcelona and Real Madrid 2026/27 Gift Pack – Home Kids Cheap Football Kits – LAMINE YAMAL 10 and MBAPPÉ 10 (With socks)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -3084,23 +3343,23 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>SKU (Google)</t>
+          <t>SKU variation</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>SKU 'CFS_ARG_AWLV_KD_MARADONA 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>SKU cha CFS_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_26/27 nhưng variation mang SKU khác đầu: CFS_BARRM1_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_26/27_16 (3-4 yrs) (+6)</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+          <t>Sửa SKU variation theo SKU cha (clone quên đổi)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/retro-argentina-maradona-10-away-kids-cheap-football-kit-1994-long-sleeve/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-and-real-madrid-2026-27-gift-pack-home-kids-cheap-football-kits-lamine-yamal-10-and-mbappe-10/</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
@@ -3112,53 +3371,53 @@
       <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Thấp</t>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Cao</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-30 02:09</t>
+          <t>2026-10-30 15:09</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>85613</v>
+        <v>85690</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CFS_ARG_AWLV_AD_MESSI 10_1994</t>
+          <t>CFS_BARRM_HOGP_KD_LAMINE YAMAL 10 MBAPPÉ 10_26/27</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Retro Argentina MESSI 10 Away Men Cheap Football Shirt 1994 Long Sleeve</t>
+          <t>Barcelona and Real Madrid 2026/27 Gift Pack – Home Kids Cheap Football Kits – LAMINE YAMAL 10 and MBAPPÉ 10 (With socks)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Sai cầu thủ</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Trang sản phẩm (option / tab / description)</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 71 ký tự (nên &lt;= 60)</t>
+          <t>Listing in sẵn LAMINE YAMAL 10 MBAPPÉ 10 nhưng trang vẫn cho/nhắc personalise: "Personalisation for 2 items only £16"</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Bỏ option / đoạn personalisation trên listing in sẵn</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/retro-argentina-messi-10-away-men-cheap-football-shirt-1994-long-sleeve/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-and-real-madrid-2026-27-gift-pack-home-kids-cheap-football-kits-lamine-yamal-10-and-mbappe-10/</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
@@ -3172,51 +3431,51 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-30 02:09</t>
+          <t>2026-10-30 03:22</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>85613</v>
+        <v>85634</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>CFS_ARG_AWLV_AD_MESSI 10_1994</t>
+          <t>CFS_BAR_AW_AD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Retro Argentina MESSI 10 Away Men Cheap Football Shirt 1994 Long Sleeve</t>
+          <t>Barcelona GORDON 17 Away Men Cheap Football Shirt 2026/27</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>SKU (Google)</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>SKU 'CFS_ARG_AWLV_AD_MESSI 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/retro-argentina-messi-10-away-men-cheap-football-shirt-1994-long-sleeve/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-away-men-cheap-football-shirt-2026-27/</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -3230,51 +3489,51 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-30 02:13</t>
+          <t>2026-10-30 03:27</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>85622</v>
+        <v>85642</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>CFS_ARG_AWLV_KD_MESSI 10_1994</t>
+          <t>CFS_BAR_AW_KD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Retro Argentina MESSI 10 Away Kids Cheap Football Kit 1994 Long Sleeve</t>
+          <t>Barcelona GORDON 17 Away Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 70 ký tự (nên &lt;= 60)</t>
+          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/retro-argentina-messi-10-away-kids-cheap-football-kit-1994-long-sleeve/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-away-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -3288,51 +3547,51 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-30 02:13</t>
+          <t>2026-10-30 03:31</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>85622</v>
+        <v>85652</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>CFS_ARG_AWLV_KD_MESSI 10_1994</t>
+          <t>CFS_BAR_HO_AD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Retro Argentina MESSI 10 Away Kids Cheap Football Kit 1994 Long Sleeve</t>
+          <t>Barcelona GORDON 17 Home Men Cheap Football Shirt 2026/27</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>SKU (Google)</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>SKU 'CFS_ARG_AWLV_KD_MESSI 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/retro-argentina-messi-10-away-kids-cheap-football-kit-1994-long-sleeve/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-home-men-cheap-football-shirt-2026-27/</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -3346,51 +3605,51 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-10-30 03:22</t>
+          <t>2026-10-30 03:35</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>85634</v>
+        <v>85660</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CFS_BAR_AW_AD_GORDON 17_26/27</t>
+          <t>CFS_BAR_HO_KD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Away Men Cheap Football Shirt 2026/27</t>
+          <t>Barcelona GORDON 17 Home Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Số lượng ảnh</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-away-men-cheap-football-shirt-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-home-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
@@ -3404,51 +3663,51 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-30 03:22</t>
+          <t>2026-10-30 03:39</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>85634</v>
+        <v>85670</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>CFS_BAR_AW_AD_GORDON 17_26/27</t>
+          <t>CFS_BAR_TH_AD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Away Men Cheap Football Shirt 2026/27</t>
+          <t>Barcelona GORDON 17 Third Men Cheap Football Shirt 2026/27</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>SKU (Google)</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>SKU 'CFS_BAR_AW_AD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-away-men-cheap-football-shirt-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-third-men-cheap-football-shirt-2026-27/</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -3462,25 +3721,25 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-30 03:22</t>
+          <t>2026-10-30 03:43</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>85634</v>
+        <v>85678</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CFS_BAR_AW_AD_GORDON 17_26/27</t>
+          <t>CFS_BAR_TH_KD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Away Men Cheap Football Shirt 2026/27</t>
+          <t>Barcelona GORDON 17 Third Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -3506,7 +3765,7 @@
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-away-men-cheap-football-shirt-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-third-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -3518,53 +3777,53 @@
       <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-10-30 03:27</t>
+          <t>2026-10-30 01:52</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>85642</v>
+        <v>85593</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>CFS_BAR_AW_KD_GORDON 17_26/27</t>
+          <t>CFS_ARG_AWLV_AD_MARADONA 10_1994</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Away Kids Cheap Football Kit 2026/27</t>
+          <t>Retro Argentina MARADONA 10 Away Men Cheap Football Shirt 1994 Long Sleeve</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Số lượng ảnh</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>SEO title dài 74 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-away-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/retro-argentina-maradona-10-away-men-cheap-football-shirt-1994-long-sleeve/</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
@@ -3576,27 +3835,27 @@
       <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-10-30 03:27</t>
+          <t>2026-10-30 01:52</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>85642</v>
+        <v>85593</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>CFS_BAR_AW_KD_GORDON 17_26/27</t>
+          <t>CFS_ARG_AWLV_AD_MARADONA 10_1994</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Away Kids Cheap Football Kit 2026/27</t>
+          <t>Retro Argentina MARADONA 10 Away Men Cheap Football Shirt 1994 Long Sleeve</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -3611,7 +3870,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>SKU 'CFS_BAR_AW_KD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>SKU 'CFS_ARG_AWLV_AD_MARADONA 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
@@ -3622,7 +3881,7 @@
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-away-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/retro-argentina-maradona-10-away-men-cheap-football-shirt-1994-long-sleeve/</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
@@ -3634,53 +3893,53 @@
       <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-10-30 03:27</t>
+          <t>2026-10-30 02:02</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>85642</v>
+        <v>85602</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CFS_BAR_AW_KD_GORDON 17_26/27</t>
+          <t>CFS_ARG_AWLV_KD_MARADONA 10_1994</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Away Kids Cheap Football Kit 2026/27</t>
+          <t>Retro Argentina MARADONA 10 Away Kids Cheap Football Kit 1994 Long Sleeve</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
+          <t>SEO title dài 73 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Cần người check</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-away-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/retro-argentina-maradona-10-away-kids-cheap-football-kit-1994-long-sleeve/</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -3692,53 +3951,53 @@
       <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-10-30 03:31</t>
+          <t>2026-10-30 02:02</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>85652</v>
+        <v>85602</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CFS_BAR_HO_AD_GORDON 17_26/27</t>
+          <t>CFS_ARG_AWLV_KD_MARADONA 10_1994</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Home Men Cheap Football Shirt 2026/27</t>
+          <t>Retro Argentina MARADONA 10 Away Kids Cheap Football Kit 1994 Long Sleeve</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Số lượng ảnh</t>
+          <t>SKU (Google)</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>SKU 'CFS_ARG_AWLV_KD_MARADONA 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-home-men-cheap-football-shirt-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/retro-argentina-maradona-10-away-kids-cheap-football-kit-1994-long-sleeve/</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -3750,53 +4009,53 @@
       <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-30 03:31</t>
+          <t>2026-10-30 02:09</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>85652</v>
+        <v>85613</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>CFS_BAR_HO_AD_GORDON 17_26/27</t>
+          <t>CFS_ARG_AWLV_AD_MESSI 10_1994</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Home Men Cheap Football Shirt 2026/27</t>
+          <t>Retro Argentina MESSI 10 Away Men Cheap Football Shirt 1994 Long Sleeve</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>SKU (Google)</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>SKU 'CFS_BAR_HO_AD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>SEO title dài 71 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-home-men-cheap-football-shirt-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/retro-argentina-messi-10-away-men-cheap-football-shirt-1994-long-sleeve/</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -3808,53 +4067,53 @@
       <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-30 03:31</t>
+          <t>2026-10-30 02:09</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>85652</v>
+        <v>85613</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>CFS_BAR_HO_AD_GORDON 17_26/27</t>
+          <t>CFS_ARG_AWLV_AD_MESSI 10_1994</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Home Men Cheap Football Shirt 2026/27</t>
+          <t>Retro Argentina MESSI 10 Away Men Cheap Football Shirt 1994 Long Sleeve</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>SKU (Google)</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
+          <t>SKU 'CFS_ARG_AWLV_AD_MESSI 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Cần người check</t>
+          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-home-men-cheap-football-shirt-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/retro-argentina-messi-10-away-men-cheap-football-shirt-1994-long-sleeve/</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -3866,53 +4125,53 @@
       <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-30 03:35</t>
+          <t>2026-10-30 02:13</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>85660</v>
+        <v>85622</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>CFS_BAR_HO_KD_GORDON 17_26/27</t>
+          <t>CFS_ARG_AWLV_KD_MESSI 10_1994</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Home Kids Cheap Football Kit 2026/27</t>
+          <t>Retro Argentina MESSI 10 Away Kids Cheap Football Kit 1994 Long Sleeve</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Số lượng ảnh</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>SEO title dài 70 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-home-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/retro-argentina-messi-10-away-kids-cheap-football-kit-1994-long-sleeve/</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -3924,27 +4183,27 @@
       <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-30 03:35</t>
+          <t>2026-10-30 02:13</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>85660</v>
+        <v>85622</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>CFS_BAR_HO_KD_GORDON 17_26/27</t>
+          <t>CFS_ARG_AWLV_KD_MESSI 10_1994</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Home Kids Cheap Football Kit 2026/27</t>
+          <t>Retro Argentina MESSI 10 Away Kids Cheap Football Kit 1994 Long Sleeve</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -3959,7 +4218,7 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>SKU 'CFS_BAR_HO_KD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>SKU 'CFS_ARG_AWLV_KD_MESSI 10_1994' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
@@ -3970,7 +4229,7 @@
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-home-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/retro-argentina-messi-10-away-kids-cheap-football-kit-1994-long-sleeve/</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -3982,53 +4241,53 @@
       <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-10-30 03:35</t>
+          <t>2026-10-30 03:22</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>85660</v>
+        <v>85634</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>CFS_BAR_HO_KD_GORDON 17_26/27</t>
+          <t>CFS_BAR_AW_AD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Home Kids Cheap Football Kit 2026/27</t>
+          <t>Barcelona GORDON 17 Away Men Cheap Football Shirt 2026/27</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>SKU (Google)</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
+          <t>SKU 'CFS_BAR_AW_AD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Cần người check</t>
+          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-home-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-away-men-cheap-football-shirt-2026-27/</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr">
@@ -4040,53 +4299,53 @@
       <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-30 03:39</t>
+          <t>2026-10-30 03:27</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>85670</v>
+        <v>85642</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>CFS_BAR_TH_AD_GORDON 17_26/27</t>
+          <t>CFS_BAR_AW_KD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Third Men Cheap Football Shirt 2026/27</t>
+          <t>Barcelona GORDON 17 Away Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Số lượng ảnh</t>
+          <t>SKU (Google)</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>Chỉ có 2 ảnh sản phẩm (nên ≥ 3: trước / sau / chi tiết)</t>
+          <t>SKU 'CFS_BAR_AW_KD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh</t>
+          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-third-men-cheap-football-shirt-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-away-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
@@ -4098,27 +4357,27 @@
       <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-30 03:39</t>
+          <t>2026-10-30 03:31</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>85670</v>
+        <v>85652</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>CFS_BAR_TH_AD_GORDON 17_26/27</t>
+          <t>CFS_BAR_HO_AD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Third Men Cheap Football Shirt 2026/27</t>
+          <t>Barcelona GORDON 17 Home Men Cheap Football Shirt 2026/27</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -4133,7 +4392,7 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>SKU 'CFS_BAR_TH_AD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>SKU 'CFS_BAR_HO_AD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -4144,7 +4403,7 @@
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-third-men-cheap-football-shirt-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-home-men-cheap-football-shirt-2026-27/</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
@@ -4156,53 +4415,53 @@
       <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-30 03:39</t>
+          <t>2026-10-30 03:35</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>85670</v>
+        <v>85660</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>CFS_BAR_TH_AD_GORDON 17_26/27</t>
+          <t>CFS_BAR_HO_KD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Third Men Cheap Football Shirt 2026/27</t>
+          <t>Barcelona GORDON 17 Home Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>SKU (Google)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
+          <t>SKU 'CFS_BAR_HO_KD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>Cần người check</t>
+          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-third-men-cheap-football-shirt-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-home-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
@@ -4214,27 +4473,27 @@
       <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-10-30 03:43</t>
+          <t>2026-10-30 03:39</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>85678</v>
+        <v>85670</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>CFS_BAR_TH_KD_GORDON 17_26/27</t>
+          <t>CFS_BAR_TH_AD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Barcelona GORDON 17 Third Kids Cheap Football Kit 2026/27</t>
+          <t>Barcelona GORDON 17 Third Men Cheap Football Shirt 2026/27</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -4249,7 +4508,7 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>SKU 'CFS_BAR_TH_KD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>SKU 'CFS_BAR_TH_AD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
@@ -4260,7 +4519,7 @@
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-third-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-gordon-17-third-men-cheap-football-shirt-2026-27/</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr">
@@ -4272,7 +4531,7 @@
       <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -4297,22 +4556,22 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Option badge</t>
+          <t>SKU (Google)</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
+          <t>SKU 'CFS_BAR_TH_KD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Cần người check</t>
+          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -4330,7 +4589,7 @@
       <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -4388,7 +4647,7 @@
       <c r="N30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -4448,7 +4707,7 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4510,7 +4769,7 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4572,7 +4831,7 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4634,7 +4893,7 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4696,7 +4955,7 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4758,7 +5017,7 @@
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4820,7 +5079,7 @@
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cần xác nhận</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">

</xml_diff>